<commit_message>
P: generador de productos (PDF con Playwright, capturas de las hojas y del PDF en WebP), PDFs y capturas generados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W9takBgfPkU2UgntoJrupH
</commit_message>
<xml_diff>
--- a/proyectos/p-webs-adsense/fabrica/productos/pack-despido/pack-despido-finiquito.xlsx
+++ b/proyectos/p-webs-adsense/fabrica/productos/pack-despido/pack-despido-finiquito.xlsx
@@ -105,7 +105,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00 &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy;;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -215,12 +215,18 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3B57"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000B1F17"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000B1F17"/>
+      <color rgb="001F3B57"/>
       <sz val="10"/>
     </font>
     <font>
@@ -439,26 +445,25 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="20" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="20" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -468,7 +473,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -489,7 +494,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -518,7 +523,7 @@
     <xf numFmtId="165" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -527,7 +532,7 @@
     <xf numFmtId="1" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="20" fillId="6" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1558,15 +1563,10 @@
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="6" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="20" customHeight="1">
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t>Amarillo</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Escribe tú en las celdas amarillas. Las demás se calculan solas: no hace falta tocarlas.</t>
+          <t>✎  Las celdas amarillas las rellenas tú; el resto se calcula solo.</t>
         </is>
       </c>
     </row>
@@ -1910,15 +1910,10 @@
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="20" customHeight="1">
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t>Amarillo</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Escribe tú en las celdas amarillas. Las demás se calculan solas: no hace falta tocarlas.</t>
+          <t>✎  Las celdas amarillas las rellenas tú; el resto se calcula solo.</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2070,7 @@
     <row r="16">
       <c r="B16" s="36" t="inlineStr">
         <is>
-          <t>Último día para presentar la papeleta de conciliación</t>
+          <t>Último día para la papeleta</t>
         </is>
       </c>
       <c r="C16" s="37">

</xml_diff>